<commit_message>
Source Data: trading-unit labels and sector-fuel dots (Fig. 1), first justified cost year and CO2 above the axis (Fig. 4), no-net-trade flag (Fig. 5); fuller READMEs
</commit_message>
<xml_diff>
--- a/source_data/Fig1.xlsx
+++ b/source_data/Fig1.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="box_statistics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cell_costs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demand_by_route" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sector_fuel_map" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +452,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Box plots: 1st, 25th, 50th, 75th and 99th percentiles across the 2,740 land cells of each cell's median levelized cost over 20 weather years; US$ per MMBtu, lower heating value</t>
+          <t>Middle, box plots: 1st, 25th, 50th, 75th and 99th percentiles across the 2,740 land cells of each cell's median levelized cost over 20 weather years; US$ per MMBtu, lower heating value. trading_unit_median_iqr is the label under each box: median (interquartile range) in the unit in which the fuel is traded</t>
         </is>
       </c>
     </row>
@@ -475,17 +476,41 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bar: addressable demand of the 139 economies by production route, billion MMBtu per year; marine fuel counted 70% methanol and 30% ammonia</t>
+          <t>Right, bar: addressable demand of the 139 economies by production route, billion MMBtu per year (total 76.1), and its share in percent; marine fuel counted 70% methanol and 30% ammonia</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>sector_fuel_map</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Right, dots: the fuels that can serve each end use sector</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The production chain (left) is a schematic; its model is described in the Methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>work/caselow/2025mid/data (lcoh_global_&lt;year&gt;_reg.csv, co2_cost_by_cell.csv, global_trajectory_countries.csv); code lcof.fig_main_framework</t>
         </is>
@@ -502,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,6 +561,11 @@
           <t>p99_usd_mmbtu</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>trading_unit_median_iqr</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -558,6 +588,11 @@
       <c r="F2" t="n">
         <v>163.58</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>US$6.5/kg (5.2-8.4)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -580,6 +615,11 @@
       <c r="F3" t="n">
         <v>202.38</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>US$1,349/t (1,081-1,737)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -602,6 +642,11 @@
       <c r="F4" t="n">
         <v>234.92</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>US$85/MMBtu (68-106)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -624,6 +669,11 @@
       <c r="F5" t="n">
         <v>225.54</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>US$1,548/t (1,232-1,939)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -646,6 +696,11 @@
       <c r="F6" t="n">
         <v>279.03</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>US$558/bbl (451-692)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -667,6 +722,11 @@
       </c>
       <c r="F7" t="n">
         <v>249.97</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>US$6.90/gal (5.48-8.62)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -102219,4 +102279,126 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>agriculture</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ammonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>buildings + industry</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>e-methane</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>buildings + industry</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>e-jet / e-diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>chemicals + shipping</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>methanol</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>chemicals + shipping</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ammonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>aviation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>e-jet / e-diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>road transport</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ethanol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>road transport</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>e-jet / e-diesel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>